<commit_message>
Add Article 240 rules to reglas_normativas (protección contra sobrecorriente)
Adds R-009 to R-017: conductor protection and standard breaker/fuse
sizes, parallel devices, thermal devices, ground-fault protection for
large services, tap/location rules, and field-verifiable placement
requirements (accessibility, height, prohibited locations, mounting
position).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reglas-normativas/reglas_normativas.xlsx
+++ b/reglas-normativas/reglas_normativas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Reglas Normativas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tabla Ampacidad 310-15b16" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reglas Normativas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla Ampacidad 310-15b16" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -847,6 +847,384 @@
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>R-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>240-4</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Proteccion de conductores segun ampacidad</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Se esta seleccionando el dispositivo de proteccion contra sobrecorriente (fusible o interruptor) de cualquier conductor que no sea cordon flexible, cable flexible ni alambre de luminaria.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>El valor nominal del dispositivo de proteccion no debe exceder la ampacidad del conductor determinada segun el Articulo 310-15 (ya corregida por temperatura y agrupamiento), salvo las excepciones de 240-4(a) a (g) (redondeo al valor estandar superior para protecciones &lt;=800A, topes para conductores pequenos, etc.).</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Calculo de ampacidad corregida del conductor + valor nominal del dispositivo elegido, mostrando que uno no excede al otro (o citando la excepcion aplicable de 240-4).</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 240-4</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>R-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>240-6(a)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Capacidades estandar de fusibles e interruptores</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Se necesita expresar la proteccion contra sobrecorriente como un valor comercial (no un valor calculado arbitrario).</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>El valor nominal debe tomarse de la lista de capacidades estandar de la Tabla 240-6(a): 15, 20, 25, 30, 35, 40, 45, 50, 60, 70, 80, 90, 100, 110, 125, 150, 175, 200, 225, 250, 300, 350, 400, 450, 500, 600, 700, 800, 1000, 1200, 1600, 2000, 2500, 3000 A (mas 1, 3, 6, 10 y 601 A solo para fusibles).</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Valor nominal del dispositivo especificado en el proyecto, verificado contra la lista de la Tabla 240-6(a).</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 240-6(a), Tabla 240-6(a)</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>R-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>240-8</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Fusibles o interruptores en paralelo</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>El diseno propone dos o mas fusibles o interruptores automaticos individuales conectados en paralelo para aumentar la capacidad de proteccion.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>NO se permite conectar en paralelo fusibles individuales, interruptores automaticos o combinaciones de ellos, salvo que esten ensamblados en paralelo de fabrica y aprobados como una sola unidad.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Ficha tecnica/listado del fabricante que confirme que el dispositivo es un ensamble aprobado como unidad, si se usa esta configuracion.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 240-8</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>R-012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>240-9</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Dispositivos termicos no sustituyen proteccion contra sobrecorriente</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Se esta considerando un relevador termico u otro dispositivo que no esta disenado para abrir cortocircuitos o fallas a tierra como proteccion contra sobrecorriente del conductor.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Los dispositivos termicos NO deben usarse para proteccion contra sobrecorriente por cortocircuito o falla a tierra. Excepcion: se permite su uso para proteger contra SOBRECARGA los conductores del circuito derivado de un motor, si cumplen 430-40.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Especificacion del dispositivo de proteccion contra cortocircuito/falla a tierra independiente del relevador termico (salvo caso de motor bajo 430-40).</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 240-9</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>R-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>240-13</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Proteccion de falla a tierra en acometidas/alimentadores grandes</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>El sistema es en estrella, solidamente puesto a tierra, con mas de 150 V a tierra pero no mas de 1000 V entre fases, y el medio principal de desconexion (acometida o edificio) tiene capacidad nominal de 1000 A o mayor.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Debe proporcionarse proteccion contra fallas a tierra del equipo, de acuerdo con 230-95, para cada dispositivo usado como medio principal de desconexion. No aplica a procesos industriales continuos donde un paro no ordenado incremente riesgos, instalaciones ya protegidas por otros requisitos, ni bombas contra incendio.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Memoria que muestre tension del sistema, capacidad del medio de desconexion, y especificacion del dispositivo de proteccion de falla a tierra instalado (o justificacion de excepcion aplicable).</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 240-13</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>R-014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>240-21</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Ubicacion de la proteccion contra sobrecorriente</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Se esta definiendo en que punto del circuito se instala el dispositivo de proteccion contra sobrecorriente.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>La proteccion debe ubicarse en el punto donde el conductor recibe su alimentacion (origen del circuito), salvo las excepciones de derivaciones/taps de 240-21(a) a (h) (p. ej. derivaciones no mayores a 3.00 m que cumplan ampacidad minima y esten en canalizacion, entre otras condiciones especificas por tipo de derivacion).</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Diagrama unifilar o plano que muestre la ubicacion del dispositivo de proteccion respecto al origen del conductor; si se usa una excepcion de derivacion, memoria que confirme el cumplimiento de las condiciones especificas de esa excepcion (longitud, ampacidad minima, canalizacion, etc.).</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 240-21</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>R-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>240-24(a)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Accesibilidad y altura de dispositivos de sobrecorriente</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Se esta definiendo la ubicacion fisica de un interruptor o interruptor automatico en la instalacion.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>El dispositivo debe quedar facilmente accesible, y el centro de la manija de operacion, en su posicion mas alta, no debe quedar a mas de 2.00 m sobre el piso o plataforma de trabajo (salvo las excepciones de 240-24(a)(1) a (4): electroductos, proteccion suplementaria, dispositivos de acometida segun 225-40/230-92, o acceso por medios portatiles junto al equipo que alimentan).</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Plano o verificacion en sitio de la altura de montaje del centro de la manija del dispositivo (medicion en metros desde el piso terminado).</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 240-24(a)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>R-016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>240-24(c-f)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Ubicaciones prohibidas para dispositivos de sobrecorriente</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Se esta eligiendo el sitio donde se instalara un interruptor, interruptor automatico o centro de carga.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>El dispositivo NO debe quedar: (c) expuesto a dano fisico; (d) cerca de material facilmente inflamable (p. ej. closets de ropa); (e) dentro de cuartos de bano, en unidades de vivienda, dormitorios o habitaciones/suites de huesped; (f) sobre los peldanos de una escalera.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Fotografia o plano de la ubicacion final del tablero/interruptor mostrando que no incurre en ninguna de las 4 condiciones prohibidas.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 240-24, incisos c), d), e) y f)</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>R-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>240-33</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Posicion de las envolventes de proteccion</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Se esta instalando la envolvente (gabinete) de un dispositivo de proteccion contra sobrecorriente.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>La envolvente debe instalarse en posicion VERTICAL, a menos que se demuestre que es impractico. Excepcion: se permite horizontal si el interruptor automatico esta instalado conforme a 240-81 (interruptores especificamente disenados/aprobados para montaje horizontal).</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Fotografia o verificacion en sitio de la orientacion de montaje del gabinete/centro de carga.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 240-33</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Borrador</t>
         </is>

</xml_diff>

<commit_message>
Add Article 220 rules and demand-factor tables (cálculo de cargas)
Adds R-018 to R-028: minimum lighting load per m2, receptacle loads,
the dwelling double-count rule, 125% largest-motor rule, demand factors
for general lighting and non-dwelling receptacles, fixed heating,
small-appliance/laundry circuits, 75% fixed-appliance factor,
non-coincident loads and neutral sizing.

Also adds a "Tablas Art 220" sheet with Tables 220-12, 220-42, 220-44
and 220-54 digitized for later use in the calculator.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reglas-normativas/reglas_normativas.xlsx
+++ b/reglas-normativas/reglas_normativas.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reglas Normativas" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla Ampacidad 310-15b16" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tablas Art 220" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +41,11 @@
       <name val="Arial"/>
       <i val="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -82,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -96,6 +102,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -461,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1225,6 +1232,468 @@
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>R-018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>220-12</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Carga minima de alumbrado general por m2</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Se esta calculando la carga de alumbrado general de un inmueble (cualquier tipo: vivienda, oficina, escuela, tienda, etc.).</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>La carga minima debe ser &gt;= la carga unitaria en VA/m2 de la Tabla 220-12 segun el tipo de inmueble (ver hoja 'Tablas Art 220'), multiplicada por el area del piso calculada con dimensiones EXTERIORES del edificio. En vivienda no se cuentan patios abiertos, cocheras ni espacios sin terminar no adaptables.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Plano con el area de piso por nivel (m2, dimensiones exteriores), tipo de inmueble declarado, y la carga de alumbrado general resultante en VA.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 220-12, Tabla 220-12</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>R-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>220-14(i)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Carga por salida de contacto</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Se esta calculando la carga de salidas de contactos de uso general (fuera de vivienda, o en vivienda cuando no aplica 220-14(j)).</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Cada contacto sencillo o multiple montado en el mismo yugo se calcula con minimo 180 VA. Un contacto multiple de cuatro o mas contactos se calcula con minimo 90 VA por cada contacto.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Conteo de salidas de contacto por circuito/tablero y la carga en VA asignada a cada una.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 220-14(i)</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>R-020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>220-14(j)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Contactos en vivienda ya incluidos en alumbrado general</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>El inmueble es vivienda unifamiliar, bifamiliar, multifamiliar, o habitacion/suite de huespedes de hotel o motel.</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>NO se debe sumar carga adicional por las salidas de contactos de uso general de 20 A o menos ni por las salidas de alumbrado de 210-70: ya estan incluidas en la carga de alumbrado general calculada con 220-12 (Tabla 220-12, 33 VA/m2 para vivienda). Sumarlas aparte es un error de doble conteo.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Memoria de calculo que muestre que la carga de contactos de uso general no se sumo por separado a los VA/m2 de alumbrado general.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 220-14(j)</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>R-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>220-18(a)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Carga total con motores: 125% del motor mayor</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Un circuito alimenta equipo accionado por motor fijo en sitio de mas de 93.25 W (1/8 HP) en combinacion con otras cargas.</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>La carga total calculada debe basarse en 125% de la carga del motor MAS GRANDE, mas la suma de las otras cargas (los demas motores y cargas se suman al 100%). Si el circuito alimenta SOLO motores aplica el Art. 430; si alimenta solo aire acondicionado/refrigeracion aplica el Art. 440.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Memoria que identifique el motor mas grande del circuito, el 125% aplicado a el, y la suma del resto de cargas al 100%.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 220-18(a)</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>R-022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>220-42</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Factores de demanda de alumbrado general</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Se esta calculando la carga de un ALIMENTADOR o ACOMETIDA (no de un circuito derivado) y ya se tiene la carga de alumbrado general.</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Aplicar los factores de demanda de la Tabla 220-42 por escalones segun tipo de inmueble (ver hoja 'Tablas Art 220'). Ej. vivienda: 100% de los primeros 3000 VA, 35% de 3001 a 120000 VA, 25% del excedente. ATENCION: estos factores NO se deben aplicar para determinar el NUMERO de circuitos derivados de alumbrado.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Memoria con la carga de alumbrado general antes y despues de aplicar la demanda, mostrando el desglose por escalones y el tipo de inmueble usado.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 220-42, Tabla 220-42</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>R-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>220-44</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Factores de demanda de contactos (no vivienda)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Se calcula el alimentador/acometida de un inmueble que NO es vivienda y se tiene la carga de contactos calculada con 220-14(h) e (i).</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Se permite aplicar los factores de demanda de la Tabla 220-44: 100% de los primeros 10 kVA y 50% del excedente. Alternativamente se pueden aplicar los factores de la Tabla 220-42.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Memoria con la carga total de contactos y el desglose del factor de demanda aplicado (primeros 10 kVA al 100%, resto al 50%).</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 220-44, Tabla 220-44</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>R-024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>220-51</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Calefaccion electrica fija de ambiente</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>El inmueble tiene calefaccion electrica fija de ambiente.</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>La carga se calcula al 100% de la carga total conectada (sin factor de demanda). Ademas, la corriente nominal de la acometida/alimentador nunca debe ser menor al valor nominal del circuito derivado mas grande que alimenta. Excepcion: se permite menos del 100% si los equipos operan por ciclos o no todos a la vez, siempre que los conductores tengan ampacidad para la carga asi calculada.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Listado de equipos de calefaccion con su capacidad nominal, carga total al 100%, y comparacion contra el circuito derivado mayor.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 220-51</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>R-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>220-52</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Circuitos de aparatos pequenos y lavadora en vivienda</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Unidad de vivienda MAYOR a 60 m2 (la seccion no aplica a viviendas de 60 m2 o menos).</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Debe incluirse 1500 VA por cada circuito derivado de 2 hilos para aparatos pequenos (210-11(c)(1)) y 1500 VA por cada circuito derivado de 2 hilos para lavadora (210-11(c)(2)). Estas cargas pueden incluirse junto con la de alumbrado general y aplicarles los factores de demanda de la Tabla 220-42.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Memoria que liste los circuitos de aparatos pequenos y de lavadora considerados, con 1500 VA asignados a cada uno.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 220-52</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>R-026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>220-53</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Factor de demanda para aparatos fijos en vivienda</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Vivienda unifamiliar, bifamiliar o multifamiliar con CUATRO O MAS aparatos fijos conectados al mismo alimentador.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Se permite aplicar un factor de demanda del 75% a la suma de las capacidades de placa de datos de esos aparatos. NO se incluyen en este 75%: estufas electricas, secadoras de ropa, equipo de calefaccion electrica ni aire acondicionado (esos tienen sus propias reglas).</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Listado de aparatos fijos con su capacidad de placa, conteo (&gt;=4) y el 75% aplicado, dejando fuera estufas, secadoras, calefaccion y A/A.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 220-53</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>R-027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>220-60</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Cargas no coincidentes</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>El alimentador o acometida alimenta dos o mas cargas que no es probable que operen simultaneamente (p. ej. calefaccion y aire acondicionado).</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Se permite omitir del calculo la MENOR de las dos cargas no coincidentes.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Justificacion tecnica de por que las cargas no pueden ser simultaneas, e indicacion de cual se omitio del calculo.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 220-60</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>R-028</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>220-61</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Carga del neutro del alimentador o acometida</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Se esta dimensionando el conductor neutro de un alimentador o acometida.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>La carga del neutro es el MAXIMO DESEQUILIBRIO: la carga neta maxima calculada entre el neutro y cualquier conductor de fase. Reduccion permitida: factor adicional de 70% sobre la parte correspondiente a estufas/secadoras (Tablas 220-54 y 220-55) y sobre la parte del desequilibrio que exceda 200 A. PROHIBIDO reducir: en circuitos de 3 hilos formados por neutro + 2 fases de un sistema 3F-4H estrella, y en la parte que alimente cargas NO LINEALES en sistemas 3F-4H estrella (ahi el neutro puede requerir incluso mayor capacidad por armonicas).</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Memoria de calculo del desequilibrio maximo, con las reducciones aplicadas o la justificacion de por que no se redujo (cargas no lineales, sistema estrella 3F-4H).</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 220-61</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Borrador</t>
         </is>
@@ -2123,4 +2592,587 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Tabla 220-12.- Cargas de alumbrado general por tipo de inmueble</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Tipo de inmueble</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Carga unitaria (VA/m2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Casas de huespedes</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Clubes</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Cuarteles y auditorios</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Depositos (almacenamiento)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Edificios de oficinas</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Edificios industriales y comerciales (lugares de almacenamiento)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Escuelas</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Estacionamientos comerciales</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Hospitales</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Hoteles y moteles, incluidos apartamentos sin cocineta</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Iglesias</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Juzgados</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Peluquerias y salones de belleza</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Restaurantes</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Tiendas</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Unidades de vivienda (ver 220-14(j))</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Vestibulos, pasillos, closets, escaleras (excepto vivienda)</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Lugares de reunion y auditorios (excepto vivienda)</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Bodegas (excepto vivienda)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Tabla 220-42.- Factores de demanda de cargas de alumbrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>Tipo de inmueble</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>Parte de la carga (VA)</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>Factor de demanda (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Almacenes</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Primeros 12,500 o menos</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Almacenes</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>A partir de 12,500</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Hospitales*</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Primeros 50,000 o menos</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Hospitales*</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>A partir de 50,000</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Hoteles y moteles (incl. apartamentos sin cocina)*</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Primeros 20,000 o menos</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Hoteles y moteles (incl. apartamentos sin cocina)*</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>De 20,001 a 100,000</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Hoteles y moteles (incl. apartamentos sin cocina)*</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>A partir de 100,000</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Unidades de vivienda</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Primeros 3,000 o menos</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Unidades de vivienda</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>De 3,001 a 120,000</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Unidades de vivienda</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>A partir de 120,000</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Todos los demas</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Voltamperes totales</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>* No aplicar estos factores a alimentadores de zonas donde puede usarse todo el alumbrado al mismo tiempo (quirofanos, comedores, salones de baile).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Tabla 220-44.- Factores de demanda para contactos (inmuebles que NO son vivienda)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>Parte de la carga de contactos (VA)</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>Factor de demanda (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Primeros 10 kVA o menos</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>A partir de 10 kVA</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Tabla 220-54.- Factores de demanda para secadoras domesticas de ropa</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>Numero de secadoras</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>Factor de demanda (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Carga minima por secadora: 5000 VA o la placa de datos, la que sea mayor (Art. 220-54).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="A39:C39"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Article 250 rules and grounding tables (puesta a tierra)
Adds R-029 to R-038: grounding electrode requirements (rod/pipe length
and diameter, mandatory supplemental electrode with the 25-ohm
exception, minimum spacing, concrete-encased electrode), grounding
electrode conductor sizing, and equipment grounding conductor sizing —
including 250-122(b), which requires the ground conductor to be scaled
up whenever phase conductors are upsized (as ElectroNOM does for
voltage drop).

Also adds a "Tablas Art 250" sheet with Tables 250-66 and 250-122
digitized.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reglas-normativas/reglas_normativas.xlsx
+++ b/reglas-normativas/reglas_normativas.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reglas Normativas" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla Ampacidad 310-15b16" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tablas Art 220" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tablas Art 250" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1694,6 +1695,426 @@
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>R-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>250-52(a)(5)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Electrodos de varilla y tubería</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Se usara una varilla o tubo como electrodo de puesta a tierra.</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>El electrodo debe tener minimo 2.44 m de longitud. Si es tubo/tubo conduit, no menor a designacion 21 (tamano comercial 3/4) y si es de acero debe estar galvanizado o con otro recubrimiento contra corrosion. Si es varilla de acero inoxidable o acero recubierto de cobre o zinc, minimo 16 mm de diametro. El electrodo debe estar libre de recubrimientos no conductores (pintura, esmalte).</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Ficha tecnica/factura del electrodo (longitud, diametro, material y recubrimiento) y fotografia de la instalacion antes del relleno.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 250-52(a)(5) y 250-53(a)(1)</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>R-030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>250-53(a)(2)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Electrodo complementario obligatorio</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>El sistema de puesta a tierra se resolvera con UN SOLO electrodo de varilla, tubería o placa.</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Un solo electrodo de varilla, tubería o placa DEBE complementarse con un electrodo adicional de los tipos de 250-52(a)(2) a (a)(8). EXCEPCION: no se requiere el electrodo adicional si se mide y demuestra que la resistencia a tierra del electrodo unico es de 25 ohms o menos.</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Reporte de medicion de resistencia a tierra (telurometro) con valor &lt;= 25 ohms, o evidencia fotografica del segundo electrodo instalado y conectado.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 250-53(a)(2) y su Excepcion</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>R-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>250-53(a)(3)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Separación mínima entre electrodos</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Se instalaran dos o mas electrodos de varilla, tubería o placa.</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Los electrodos deben estar separados cuando menos 1.80 m entre si. NOTA de la norma: la eficiencia aumenta separandolos 2 veces la longitud de la varilla mas larga (p. ej. ~4.9 m para varillas de 2.44 m). Ademas, cada electrodo debe estar a no menos de 1.80 m de electrodos de otros sistemas de puesta a tierra (incluidos pararrayos).</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Plano o croquis acotado de la ubicacion de los electrodos mostrando la separacion real en metros.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 250-53(a)(3) y 250-53(b)</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>R-032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>250-52(a)(3)</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Electrodo recubierto en concreto (tipo Ufer)</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Se aprovechara el acero de refuerzo de la cimentacion como electrodo de puesta a tierra.</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Debe consistir en al menos 6.00 m de: varilla de refuerzo de acero desnuda o galvanizada de minimo 13 mm de diametro (continua o unida por amarre/soldadura), O conductor de cobre desnudo de minimo 21.2 mm2 (4 AWG). Los componentes deben tener minimo 5 cm de recubrimiento de concreto y estar horizontales en la cimentacion o zapata en contacto DIRECTO con la tierra (no cuenta si hay aislante, barrera de vapor o pelicula que separe el concreto del suelo).</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Fotografias de la armadura/conductor antes del colado, mostrando longitud, diametro y la conexion; nota en plano de cimentacion.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 250-52(a)(3)</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>R-033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>250-66</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Tamaño del conductor del electrodo de puesta a tierra</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Se dimensiona el conductor que va del sistema al electrodo de puesta a tierra (en acometida, edificio alimentado, o sistema derivado separado).</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>El tamano no debe ser menor al de la Tabla 250-66, segun el mayor conductor de entrada de acometida (ver hoja 'Tablas Art 250'). TOPES: si el conductor conecta UNICAMENTE a electrodos de varilla, tubería o placa, no se exige mayor a 13.3 mm2 (6 AWG) de cobre o 21.2 mm2 (4 AWG) de aluminio; si conecta unicamente a electrodo recubierto de concreto, no se exige mayor a 21.2 mm2 (4 AWG) de cobre.</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Memoria con el calibre del mayor conductor de acometida, el calibre resultante de la Tabla 250-66 y el tope aplicado si corresponde.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 250-66, Tabla 250-66</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>R-034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>250-122(a)</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Tamaño del conductor de puesta a tierra de equipos</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Se dimensiona el conductor de puesta a tierra de equipos (tierra fisica del circuito) de cualquier circuito derivado o alimentador.</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>El calibre no debe ser menor al de la Tabla 250-122, entrando con la CAPACIDAD DEL DISPOSITIVO DE PROTECCION del circuito (no con la corriente) — ver hoja 'Tablas Art 250'. Pero en ningun caso se exige que sea mayor que los conductores de fase del circuito.</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Memoria que muestre el interruptor del circuito, el calibre de tierra obtenido de la Tabla 250-122 y la verificacion de que no excede el calibre de fase.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 250-122(a), Tabla 250-122</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>R-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>250-122(b)</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Aumento proporcional del conductor de tierra</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Se aumento el calibre de los conductores de fase por encima del minimo requerido por ampacidad (caso tipico: se subio de calibre para cumplir el 3% de caida de tension en un circuito largo).</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>El conductor de puesta a tierra de equipos tipo alambre DEBE aumentarse proporcionalmente al area (mm2 o kcmil) en que se aumentaron los conductores de fase. Ejemplo: si la fase paso de 10 AWG (5.26 mm2) a 8 AWG (8.37 mm2), factor = 8.37/5.26 = 1.59, y el area de tierra minima de tabla debe multiplicarse por ese factor.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Memoria con: calibre de fase minimo por ampacidad, calibre de fase finalmente adoptado, factor de aumento calculado, y calibre de tierra resultante.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 250-122(b)</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>R-036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>250-122(c)</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Tierra única para circuitos múltiples</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Un solo conductor de puesta a tierra de equipos se instalara para varios circuitos que comparten la misma canalizacion, cable o charola.</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Ese conductor unico debe dimensionarse con base en el MAYOR dispositivo de proteccion contra sobrecorriente presente en esa canalizacion, cable o charola.</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Listado de circuitos que comparten la canalizacion con sus interruptores, identificando el mayor, y el calibre de tierra resultante de la Tabla 250-122.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 250-122(c)</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>R-037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>250-124(b)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Prohibido interrumpir el conductor de tierra</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Se esta disenando el sistema de desconexion de un circuito o equipo.</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>NO se debe colocar ningun cortacircuito automatico ni desconectador en el conductor de puesta a tierra de equipos, a menos que su apertura desconecte TODAS las fuentes de alimentacion. La tierra debe permanecer continua.</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Diagrama unifilar que muestre el conductor de puesta a tierra sin dispositivos de interrupcion en su trayectoria.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 250-124(b)</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>R-038</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>250-126</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Identificación de la terminal de tierra</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Se instalan dispositivos (contactos, apagadores, equipos) con terminal para conductor de puesta a tierra.</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>La terminal de conexion del conductor de puesta a tierra de equipos debe identificarse por: (1) tornillo con cabeza de color VERDE no facilmente removible, (2) tuerca de color VERDE no facilmente removible, o (3) el simbolo de puesta a tierra indicado en la Figura 250-126.</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Fotografia o ficha del dispositivo mostrando la identificacion verde o el simbolo de tierra en la terminal.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>NOM-001-SEDE-2018, Articulo 250-126</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Borrador</t>
         </is>
@@ -3175,4 +3596,534 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Tabla 250-66.- Conductor del electrodo de puesta a tierra (sistemas de corriente alterna)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Mayor conductor de acometida - Cobre</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Mayor conductor de acometida - Aluminio</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Conductor al electrodo - Cobre</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Conductor al electrodo - Aluminio</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2 AWG o menor (33.6 mm2)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>1/0 AWG o menor (53.5 mm2)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>8 AWG (8.37 mm2)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>6 AWG (13.3 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1 o 1/0 AWG (42.4 o 53.5 mm2)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2/0 o 3/0 AWG (67.4 o 85.0 mm2)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>6 AWG (13.3 mm2)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>4 AWG (21.2 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2/0 o 3/0 AWG (67.4 o 85.0 mm2)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>4/0 AWG o 250 kcmil (107 o 127 mm2)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>4 AWG (21.2 mm2)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2 AWG (33.6 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Mas de 3/0 a 350 kcmil</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Mas de 250 a 500 kcmil</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2 AWG (33.6 mm2)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1/0 AWG (53.5 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Mas de 350 a 600 kcmil</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Mas de 500 a 900 kcmil</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>1/0 AWG (53.5 mm2)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>3/0 AWG (85.0 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Mas de 600 a 1100 kcmil</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Mas de 900 a 1750 kcmil</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2/0 AWG (67.4 mm2)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>4/0 AWG (107 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Mas de 1100 kcmil</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Mas de 1750 kcmil</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>3/0 AWG (85.0 mm2)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>250 kcmil (127 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Topes (250-66 a,b,c): si el conductor va UNICAMENTE a varilla/tubería/placa, no se exige mayor a 6 AWG Cu / 4 AWG Al. Si va unicamente a electrodo recubierto de concreto, no se exige mayor a 4 AWG Cu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Tabla 250-122.- Tamaño mínimo del conductor de puesta a tierra de equipos</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Capacidad del dispositivo de protección (A), sin exceder</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>Cobre</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>Aluminio o Al recubierto de Cu</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>14 AWG (2.08 mm2)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>12 AWG</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>12 AWG (3.31 mm2)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>10 AWG</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>10 AWG (5.26 mm2)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>8 AWG</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>8 AWG (8.37 mm2)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>6 AWG</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>6 AWG (13.3 mm2)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>4 AWG (21.2 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>4 AWG (21.2 mm2)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>2 AWG (33.6 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>3 AWG (26.7 mm2)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>1 AWG (42.4 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2 AWG (33.6 mm2)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>1/0 AWG (53.5 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>1 AWG (42.4 mm2)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>2/0 AWG (67.4 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>800</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>1/0 AWG (53.5 mm2)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>3/0 AWG (85.0 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>2/0 AWG (67.4 mm2)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>4/0 AWG (107 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>3/0 AWG (85.0 mm2)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>250 kcmil (127 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>1600</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>4/0 AWG (107 mm2)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>350 kcmil (177 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>250 kcmil (127 mm2)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>400 kcmil (203 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>350 kcmil (177 mm2)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>600 kcmil (304 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>400 kcmil (203 mm2)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>600 kcmil (304 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>500 kcmil (253 mm2)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>750 kcmil (380 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>700 kcmil (355 mm2)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>1200 kcmil (608 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>6000</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>800 kcmil (405 mm2)</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>1200 kcmil (608 mm2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Se entra a esta tabla con la CAPACIDAD DEL INTERRUPTOR, no con la corriente. El conductor de tierra nunca debe exceder el calibre de fase (250-122a), y debe aumentarse proporcionalmente si se aumento el calibre de fase (250-122b).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A11:D11"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add validation notes sheet from the CENTURA memoria review
Records three findings from comparing ElectroNOM against a real
executed project's calculation memo, kept on a separate sheet because
these are not NOM rules but discrepancies worth tracking:

- N-001: feeder D (130 m) specifies 4 AWG as the voltage-drop minimum,
  but 8 AWG already meets 3%. Two independent deviations identified:
  using the derated current for voltage drop, and an unexplained extra
  size jump. Left open pending the responsible engineer's decision.
- N-002: breaker sized to conductor table ampacity rather than to the
  design current. Resolved — the app follows Art. 240-6(a)/240-4.
- N-003: ampacity taken from the 60 C column with correction factors
  from the 75/90 C columns.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reglas-normativas/reglas_normativas.xlsx
+++ b/reglas-normativas/reglas_normativas.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla Ampacidad 310-15b16" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tablas Art 220" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tablas Art 250" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas de validación" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +48,18 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E2761"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="005A5F7A"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -89,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -104,6 +117,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4126,4 +4143,176 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Notas de validación — hallazgos al comparar ElectroNOM contra memorias de cálculo reales</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Estas notas NO son reglas normativas: son diferencias detectadas entre lo que calcula ElectroNOM (con base en la NOM-001-SEDE-2018) y lo que aparece en documentos de proyectos ya ejecutados. Sirven para decidir criterios de diseño y detectar errores de método.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Documento / circuito</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Hallazgo</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Análisis normativo</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Impacto</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="210" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>N-001</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Memoria Jardín de Eventos CENTURA (27-nov-2025) — Alimentador Centro de carga D (fuerza, contactos y alumbrado oficina). Trifásico 220 V, 4,640 W, factor de carga 0.8, FP 0.9, 130 m, ambiente 40 °C.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>El documento especifica 4 AWG de cobre para fase y neutro, presentándolo como el calibre mínimo que cumple el 3% de caída de tensión. ElectroNOM calcula que 8 AWG ya cumple (2.65%).</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Se detectaron DOS desviaciones independientes:
+1) El documento usa la CORRIENTE CORREGIDA (Icorr = 15 A) en la fórmula de caída de tensión. Esto es un error de método: los factores de temperatura (0.91) y agrupamiento (0.8) sirven para degradar la AMPACIDAD del conductor (Art. 310-15(b)(2) y (b)(3)(a)), no para inflar la corriente que realmente circula. Por el conductor pasan 10.9 A reales. Usar 15 A cuenta dos veces el castigo por derateo.
+2) Aun aceptando su propio método (15 A y su fórmula que solo usa R), el resultado debería ser 6 AWG (2.47%), no 4 AWG — el 8 AWG falla con 3.93% pero el 6 AWG pasa. El salto hasta 4 AWG no está justificado en el documento.
+La única hipótesis que aterriza exactamente en 4 AWG es haber usado 260 m (longitud total ida y vuelta) en vez de 130 m de un sentido. En trifásico eso no aplica: el factor raiz(3) ya considera la geometría del circuito; el factor 2 solo corresponde a circuitos monofásicos.
+Caída de tensión calculada con Tabla 9 (R y XL reales, FP 0.9, raiz(3), 130 m, 10.9 A): 10 AWG = 4.00% | 8 AWG = 2.65% | 6 AWG = 1.70% | 4 AWG = 1.10%.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Sobredimensionamiento de aproximadamente dos calibres respecto al mínimo normativo. NO es una condición insegura (sobra cobre, no falta), pero implica costo adicional de material en ~130 m de recorrido sobre 4 conductores.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente de decisión de César (ing. responsable): aceptar 8 AWG como mínimo normativo, o mantener 4 AWG como decisión consciente de diseño por margen para cargas futuras del alimentador de oficina.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="210" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>N-002</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Memoria Jardín de Eventos CENTURA — todos los circuitos revisados (C1, AA 5 ton, D).</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>El documento dimensiona el interruptor igualándolo a la ampacidad de tabla del conductor elegido (ej. 8 AWG -&gt; 40 A, 12 AWG -&gt; 20 A), no al siguiente valor estándar por encima de la corriente de diseño.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>El Art. 240-6(a) junto con el 240-4 establecen que la protección se selecciona para la carga real, tomando la ampacidad del conductor como LÍMITE SUPERIOR, no como valor objetivo. Para el circuito C1 (22.7 A de diseño), ElectroNOM selecciona 25 A y el documento 40 A.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Protección más holgada de lo necesario: menor sensibilidad ante sobrecargas sostenidas. Cumple la norma (no excede la ampacidad del conductor) pero no es el criterio literal del Art. 240.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Resuelto: César decidió que ElectroNOM se apegue estrictamente a la norma (Art. 240-6(a)/240-4). No se implementó el criterio alterno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="210" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>N-003</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Memoria Jardín de Eventos CENTURA — circuitos con corrección por temperatura.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>El documento mezcla columnas de temperatura: toma la ampacidad base de la columna de 60 °C pero aplica factores de corrección por temperatura de la columna de 75 °C o 90 °C (usa 0.88 y 0.91 para 40 °C).</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>La Tabla 310-15(b)(2)(a) exige que el factor de corrección corresponda a la MISMA temperatura nominal del conductor con la que se tomó la ampacidad base. Para 40 °C: columna 60 °C = 0.82, columna 75 °C = 0.88, columna 90 °C = 0.91.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Inconsistencia interna del documento de referencia. ElectroNOM usa siempre la misma columna para ambos valores, por lo que no reproduce este error.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Informativo: no requiere acción en el software. Útil como criterio de revisión al auditar memorias de terceros.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Registra N-008: valida motor de calculo contra Advanced Energy y acota alcance a baja tension
Confirma caida de tension y cortocircuito de ElectroNOM contra un tercer
proyecto real (Advanced Energy Planta 3, media tension). Ambos coinciden
con el metodo punto-a-punto de la memoria dentro de 0.15%. Se descarta la
hipotesis de error de unidades (metros vs pies) en su tabla de valores C.

Por instruccion expresa, el alcance de ElectroNOM se mantiene acotado a
baja tension (Titulo 5, <1000V); el documento se usa solo como material
de validacion, no como driver de nuevas funcionalidades de media tension.
Queda registrada como mejora pendiente (no urgente) el soporte de
conductores en paralelo en el motor de cortocircuito y caida de tension.
</commit_message>
<xml_diff>
--- a/reglas-normativas/reglas_normativas.xlsx
+++ b/reglas-normativas/reglas_normativas.xlsx
@@ -4151,7 +4151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4507,6 +4507,50 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>N-008</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Memoria Tecnica Advanced Energy Planta 3 (10-abr-2026) — Alimentadores de Transformadores 03/04/05 (2500 kVA c/u, Delta-Estrella, 34.5kV/480-277V) a tablero SWBD 3000A, 8 conductores 500 kcmil de cobre en paralelo por fase, 8 m.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Memoria Tecnica Advanced Energy Planta 3 (10-abr-2026, proyecto de media tension industrial) se uso UNICAMENTE COMO APOYO para validar el motor de calculo de ElectroNOM, por instruccion expresa de Cesar: el software se acota a BAJA TENSION (Titulo 5 de la NOM, menor a 1000 V). El proyecto Advanced Energy no es un requerimiento de alcance, es solo material de prueba.
+Se validaron dos calculos contra la memoria real (3 transformadores de 2500 kVA, Delta-Estrella, 34.5kV/480-277V, alimentando un tablero SWBD 3000A a 8 m mediante 8 conductores 500 kcmil de cobre en paralelo por fase):
+1) CAIDA DE TENSION: la memoria reporta 0.16% (500 kcmil, 8 m, 480 V). Con la formula de impedancia de ElectroNOM (Tabla 9: r=0.089, x=0.128 Ohm/km) y la corriente por conductor (375.89 A = 3007.12/8), el resultado coincide (0.1606%) solo asumiendo FP=0.8. La memoria no declara el FP usado en esa seccion especifica del documento extraido.
+2) CORTOCIRCUITO AGUAS ABAJO EN EL SWBD: la memoria usa el metodo punto-a-punto (C-value / Bussmann). ElectroNOM usa el metodo por unidad. calcularCortocircuito() no soporta conductores en paralelo nativamente, asi que se extendio manualmente (impedancia del conductor / 8) para la comparacion:
+   T03 (%Z 6.61): memoria 44.41 kA vs ElectroNOM 44.35 kA (dif. 0.14%)
+   T04 (%Z 6.72): memoria 43.70 kA vs ElectroNOM 43.66 kA (dif. 0.09%)
+   T05 (%Z 6.60): memoria 44.48 kA vs ElectroNOM 44.42 kA (dif. 0.13%)
+Coinciden dentro del margen de redondeo esperado: los dos metodos son matematicamente equivalentes.
+3) HIPOTESIS DESCARTADA (metros vs pies): el metodo punto-a-punto original (Bussmann/IEEE) usa tablas de valor C calibradas para longitud en PIES. La memoria usa L=8 directamente como METROS (mismo valor que en la caida de tension). Se probo la hipotesis de que fuera un error de unidades: si lo fuera, el calculo metrico-nativo de ElectroNOM (Tabla 9 en Ohm/km) debia dar un resultado muy distinto al de la memoria. No fue asi (coincidencia dentro de 0.15%), asi que la tabla 'Cuadro 17' de la memoria ya esta adaptada a metros. NO hay error de unidades en el documento.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Confirma que el motor de ElectroNOM (calcularCaidaTension y calcularCortocircuito, metodo por unidad) produce resultados correctos y consistentes con un metodo independiente (punto-a-punto) usado en un tercer proyecto real, fuera de la familia de documentos CENTURA.
+BRECHA DE CAPACIDAD CONFIRMADA (no es un error, es una funcionalidad ausente): calcularCortocircuito() no admite multiples conductores en paralelo por fase (Art. 310-10(h)). Para reproducir el calculo de Advanced Energy fue necesario dividir la impedancia manualmente fuera de la funcion. Los conductores en paralelo SI son un tema de baja tension (aplica en Titulo 5 tambien, no es exclusivo de media tension), asi que esta brecha sigue vigente independientemente del acotamiento de alcance.
+DECISION DE ALCANCE (instruccion expresa de Cesar, 15-ago-2026): ElectroNOM se mantiene acotado a BAJA TENSION (Titulo 5, menor a 1000 V). Todo lo de media tension que aparece en la memoria de Advanced Energy (cuchillas fusibles 34.5kV, apartarrayos, transformadores tipo estacion, Titulo 6/Capitulo 9) queda explicitamente FUERA DE ALCANCE y no se debe implementar. El documento se usa solo como material de validacion del motor de calculo en la parte que SI es baja tension (el alimentador del secundario del transformador hacia el tablero, 480V).</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Ninguna correccion requerida en el motor de calculo: los dos metodos (por unidad vs punto-a-punto) coinciden. No se hacen cambios de alcance hacia media tension.
+Queda registrado como mejora pendiente (no urgente, no solicitada aun): agregar soporte de conductores en paralelo a calcularCortocircuito() y calcularCaidaTension() para proyectos de baja tension con alimentadores grandes que usan varios conductores por fase.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>CERRADA / INFORMATIVA (15-ago-2026). El motor de calculo queda validado contra un tercer proyecto real. Alcance de ElectroNOM confirmado y documentado: solo baja tension (Titulo 5, &lt;1000V). Advanced Energy Planta 3 se usa unicamente como material de prueba, no como driver de nuevas funcionalidades de media tension.
+PENDIENTE ABIERTO (separado de esta nota, sujeto a decision futura de Cesar): soporte de conductores en paralelo por fase en el motor de cortocircuito y caida de tension.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
Registra N-009: valida caida de tension y tierra contra proyecto VERTIV en baja tension
Confirma, en un tercer proyecto real (generadores QSK60, 480V, 6
conductores 500 kcmil en paralelo por fase), que el metodo de caida de
tension de ElectroNOM funciona correctamente para conductores en
paralelo, y que la Tabla 250-122(a) de tierra es correcta hasta 2500 A.

Identifica tres capacidades de baja tension aun no implementadas:
ampacidad en charola portacable (Tabla 310-15(b)(17) + Art. 392),
verificacion termica del conductor ante cortocircuito, y llenado de
charola portacable. Ninguna requiere correccion en el motor actual.
</commit_message>
<xml_diff>
--- a/reglas-normativas/reglas_normativas.xlsx
+++ b/reglas-normativas/reglas_normativas.xlsx
@@ -4151,7 +4151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4507,6 +4507,53 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>N-009</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Memoria PIE-2026-003 VERTIV (22-abr-2026, Rev.1) — Alimentadores de generadores QSK60 (1,300 kW c/u, 480V/60Hz) al tablero colector de baja tension, 6 conductores 500 kcmil de cobre en paralelo por fase, 30 m, charola portacable tipo escalera.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Memoria de Calculo de Conductores Electricos PIE-2026-003 (VERTIV, Central de Generacion y Centro de Carga en Abasto Aislado, 22-abr-2026, Rev.1) — generadores gas natural QSK60, 1,300 kW c/u, 480V/60Hz, FP 0.8. A diferencia de Advanced Energy (N-008), este proyecto SI es baja tension (Titulo 5), por lo que aplica como material de validacion de pleno derecho, no solo como apoyo.
+COINCIDENCIAS CONFIRMADAS (2):
+1) CAIDA DE TENSION con conductores en paralelo: 6 conductores 500 kcmil de cobre por fase, 30 m, In=1,954.63 A, FP 0.8. La memoria reporta e%=0.56707%. Aplicando la formula de impedancia de ElectroNOM (calcularCaidaTension, Tabla 9: r=0.105, x=0.128 Ohm/km) con la corriente dividida entre los 6 conductores (325.77 A c/u), el resultado es 0.5669% -- coincide dentro del redondeo esperado. Segunda confirmacion independiente (la primera fue N-008 con Advanced Energy) de que dividir corriente/impedancia entre el numero de conductores en paralelo reproduce el metodo real usado en campo.
+2) CONDUCTOR DE PUESTA A TIERRA: con interruptor de 2,500 A (ajuste de tiempo largo), la memoria usa la Tabla 250-122(a) y obtiene 350 kcmil de cobre (177 mm2) como area minima requerida (suben a 500 kcmil por disponibilidad comercial, no por norma). La tabla GROUND_TABLE_250_122 de ElectroNOM tiene exactamente esa fila: maxBreaker 2500 -&gt; cu 350. Coincidencia exacta.
+CAPACIDADES AUSENTES EN ELECTRONOM CONFIRMADAS (3, todas dentro de alcance de baja tension, no se pudo validar por falta de la funcionalidad, no por error):
+3) Ampacidad en charola portacable (Tabla 310-15(b)(17) + Art. 392-80(a)(2)(b) para charola cubierta, 60% de derateo sobre la ampacidad al aire libre). ElectroNOM solo implementa la Tabla 310-15(b)(16) (tuberia/canalizacion cerrada). Son tablas y metodos de instalacion distintos.
+4) Verificacion termica del conductor ante cortocircuito (formula adiabatica I^2/A^2 * t = 0.0297 * log10[(T2+234)/(T1+234)], que da el area minima de cobre para soportar la energia de falla sin danar el aislamiento). ElectroNOM solo verifica que el INTERRUPTOR tenga capacidad interruptiva suficiente (Art. 110-9); no verifica si el conductor mismo sobrevive el calentamiento de la falla.
+5) Llenado de charola portacable (Art. 392-22). ElectroNOM solo calcula llenado de tuberia (conduit).</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Confirma, en un TERCER proyecto real y esta vez enteramente de baja tension, que:
+- El metodo de caida de tension de ElectroNOM (Tabla 9, formula de impedancia) es correcto tambien para alimentadores con multiples conductores en paralelo, si se divide la corriente entre el numero de conductores.
+- La Tabla 250-122(a) implementada en GROUND_TABLE_250_122 es correcta hasta al menos 2,500 A de proteccion.
+Identifica tres capacidades de baja tension ausentes (charola portacable para ampacidad, verificacion termica del conductor ante falla, llenado de charola). Ninguna es un error del motor: son calculos que la NOM contempla (Art. 392 para charola, formula adiabatica estandar para verificacion termica) pero que ElectroNOM no implementa todavia porque hasta ahora todos los proyectos de validacion usaban tuberia (conduit), no charola, y ninguno tenia corrientes de falla lo bastante altas para que la verificacion termica del conductor fuera el factor limitante en vez de la capacidad del interruptor.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Ninguna correccion requerida en el motor de calculo existente: las dos verificaciones que si se pudieron comparar (caida de tension con conductores en paralelo, tierra por Tabla 250-122a) coinciden con la memoria real.
+Quedan registradas como mejoras pendientes (no urgentes, sujetas a priorizacion de Cesar):
+  a) Ampacidad para instalacion en charola portacable (Tabla 310-15(b)(17) + derateos del Art. 392).
+  b) Verificacion termica (I^2t) del conductor de fase ante corriente de cortocircuito.
+  c) Llenado de charola portacable (Art. 392-22).</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>CERRADA / INFORMATIVA (18-ago-2026). Motor de calculo validado por tercera vez en un proyecto real, esta vez de baja tension pura. Caida de tension con conductores en paralelo y tabla de tierra 250-122(a) confirmadas exactas.
+PENDIENTES ABIERTOS (separados de esta nota, sujetos a decision futura de Cesar sobre prioridad): soporte de ampacidad en charola portacable, verificacion termica del conductor ante cortocircuito, y llenado de charola portacable.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
Cierra N-010: decision de Cesar de seguir estrictamente la Tabla 430-52
Cesar decidio no mantener el criterio de oficina (12 AWG/20 A estandar)
para los 4 circuitos de motor pequenos que excedian el maximo de la
Tabla 430-52, y seguir lo que calcula la norma: 15 A en los 4 casos.

Accion pendiente en el proyecto (documentos de responsiva de Cesar, no
tocados por esta herramienta): corregir el interruptor de C.C. A CT1,
CT5, CT17 y C.C. B1(3F) CT3 de 20 A a 15 A.
</commit_message>
<xml_diff>
--- a/reglas-normativas/reglas_normativas.xlsx
+++ b/reglas-normativas/reglas_normativas.xlsx
@@ -4344,6 +4344,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -4809,7 +4810,14 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>ABIERTA (23-ago-2026), pendiente del criterio de Cesar -- mismo patron que N-002/N-006: decidir si mantener el criterio de oficina (12 AWG/20 A estandar para motores pequenos) o corregir a lo que calcula estrictamente la Tabla 430-52 (15 A) en los 4 circuitos senalados. No se modifico ningun documento del proyecto -- son entregables de Cesar.
-Metodologia y script quedan documentados en la memoria de la sesion (normalizar_centura.py + validar_motores.js); los archivos temporales no se conservan entre sesiones y hay que regenerarlos si se retoma este analisis.</t>
+Metodologia y script quedan documentados en la memoria de la sesion (normalizar_centura.py + validar_motores.js); los archivos temporales no se conservan entre sesiones y hay que regenerarlos si se retoma este analisis.
+CERRADA (23-ago-2026). Decision de Cesar: seguir estrictamente lo que dice la NOM (Tabla 430-52), no el criterio de oficina.
+ACCION PENDIENTE EN EL PROYECTO (no realizada por esta herramienta -- son documentos de responsiva de Cesar): corregir el interruptor de los 4 circuitos senalados de 20 A a 15 A:
+  C.C. A, CT1  'Manejadora recamara principal'          -&gt; 15 A
+  C.C. A, CT5  'Manejadora recamara 2'                  -&gt; 15 A
+  C.C. A, CT17 'Manejadora recamara planta alta'         -&gt; 15 A
+  C.C. B1(3F), CT3 'Extractores banos hombres/mujeres'   -&gt; 15 A
+CRITERIO GENERAL QUE DEJA ESTA NOTA: para circuitos de motor, el interruptor se calcula con el porcentaje de la Tabla 430-52 segun el tipo de dispositivo (250% para interruptor de tiempo inverso en tableros termomagneticos estandar como los QO de este proyecto), NO con el criterio de oficina de usar 12 AWG/20 A por default. Motores pequenos (FLC bajo) son los que mas facilmente quedan sobredimensionados con ese habito, porque 20 A es el escalon minimo 'comodo' independientemente de que tan chico sea el motor.</t>
         </is>
       </c>
     </row>

</xml_diff>